<commit_message>
Remove an input variable for lab_blood_fasting
</commit_message>
<xml_diff>
--- a/longitudinal/data_processing_elements_longitudinal-MSC.xlsx
+++ b/longitudinal/data_processing_elements_longitudinal-MSC.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Computer\twey working files\ProPASS\MSC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A5570225-6438-485D-AB2B-BC80EBD2887A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96E93E5B-C4F7-4FEA-AF72-30623FD5EC2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{EBFE0AAE-9F6E-4351-BDB4-692162CD990C}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1330" uniqueCount="468">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1330" uniqueCount="467">
   <si>
     <t>index</t>
   </si>
@@ -1418,10 +1418,6 @@
   </si>
   <si>
     <t>m_ant_bp_dias_avg</t>
-  </si>
-  <si>
-    <t>m_cm_hours_fasting;
-m_cm_reschedule</t>
   </si>
   <si>
     <t>hba1c_mmol_mol is the only source variable without the m_ prefix. Please confirm it is delivered in the same input dataset as the other follow-up 1 variables.</t>
@@ -1770,7 +1766,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -1810,6 +1806,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2180,7 +2179,7 @@
         <v>394</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="D1" s="8" t="s">
         <v>128</v>
@@ -2242,7 +2241,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>16</v>
@@ -2277,7 +2276,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>17</v>
@@ -2301,7 +2300,7 @@
         <v>253</v>
       </c>
       <c r="N3" s="1" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="Q3" s="5"/>
     </row>
@@ -2310,7 +2309,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>18</v>
@@ -2334,10 +2333,10 @@
         <v>253</v>
       </c>
       <c r="N4" s="1" t="s">
+        <v>410</v>
+      </c>
+      <c r="P4" s="4" t="s">
         <v>411</v>
-      </c>
-      <c r="P4" s="4" t="s">
-        <v>412</v>
       </c>
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.35">
@@ -2345,7 +2344,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>19</v>
@@ -2377,7 +2376,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>20</v>
@@ -2404,25 +2403,25 @@
         <v>255</v>
       </c>
       <c r="N6" s="7" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="O6" s="4" t="s">
         <v>384</v>
       </c>
       <c r="Q6" s="4" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="R6" s="4" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="S6" s="4" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="T6" s="4" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="U6" s="4" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
     </row>
     <row r="7" spans="1:21" ht="58" x14ac:dyDescent="0.35">
@@ -2430,7 +2429,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>21</v>
@@ -2468,7 +2467,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>22</v>
@@ -2509,7 +2508,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>23</v>
@@ -2539,16 +2538,16 @@
         <v>259</v>
       </c>
       <c r="N9" s="4" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="Q9" s="4" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="R9" s="4" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="S9" s="4" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
     </row>
     <row r="10" spans="1:21" ht="188.5" x14ac:dyDescent="0.35">
@@ -2556,7 +2555,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>24</v>
@@ -2594,7 +2593,7 @@
         <v>10</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>25</v>
@@ -2632,7 +2631,7 @@
         <v>11</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>26</v>
@@ -2673,7 +2672,7 @@
         <v>12</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>27</v>
@@ -2705,7 +2704,7 @@
         <v>13</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>28</v>
@@ -2743,7 +2742,7 @@
         <v>14</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C15" s="4" t="s">
         <v>29</v>
@@ -2773,10 +2772,10 @@
         <v>259</v>
       </c>
       <c r="N15" s="4" t="s">
+        <v>414</v>
+      </c>
+      <c r="P15" s="4" t="s">
         <v>415</v>
-      </c>
-      <c r="P15" s="4" t="s">
-        <v>416</v>
       </c>
     </row>
     <row r="16" spans="1:21" ht="116" x14ac:dyDescent="0.35">
@@ -2784,7 +2783,7 @@
         <v>15</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>30</v>
@@ -2822,7 +2821,7 @@
         <v>16</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C17" s="4" t="s">
         <v>31</v>
@@ -2837,7 +2836,7 @@
         <v>252</v>
       </c>
       <c r="J17" s="4" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="K17" s="1" t="s">
         <v>249</v>
@@ -2852,7 +2851,7 @@
         <v>398</v>
       </c>
       <c r="P17" s="4" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
     </row>
     <row r="18" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
@@ -2860,7 +2859,7 @@
         <v>17</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C18" s="4" t="s">
         <v>32</v>
@@ -2898,7 +2897,7 @@
         <v>18</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>33</v>
@@ -2934,13 +2933,13 @@
         <v>290</v>
       </c>
       <c r="Q19" s="4" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="R19" s="4" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="S19" s="4" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
     </row>
     <row r="20" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
@@ -2948,7 +2947,7 @@
         <v>19</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C20" s="4" t="s">
         <v>34</v>
@@ -2986,7 +2985,7 @@
         <v>20</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C21" s="4" t="s">
         <v>35</v>
@@ -3022,13 +3021,13 @@
         <v>290</v>
       </c>
       <c r="Q21" s="4" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="R21" s="4" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="S21" s="4" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
     </row>
     <row r="22" spans="1:19" ht="58" x14ac:dyDescent="0.35">
@@ -3036,7 +3035,7 @@
         <v>21</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C22" s="4" t="s">
         <v>36</v>
@@ -3077,7 +3076,7 @@
         <v>22</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C23" s="4" t="s">
         <v>37</v>
@@ -3115,7 +3114,7 @@
         <v>23</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C24" s="4" t="s">
         <v>38</v>
@@ -3151,13 +3150,13 @@
         <v>290</v>
       </c>
       <c r="Q24" s="4" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="R24" s="4" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="S24" s="4" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
     </row>
     <row r="25" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
@@ -3165,7 +3164,7 @@
         <v>24</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C25" s="4" t="s">
         <v>39</v>
@@ -3203,7 +3202,7 @@
         <v>25</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C26" s="4" t="s">
         <v>40</v>
@@ -3233,22 +3232,22 @@
         <v>265</v>
       </c>
       <c r="N26" s="4" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="O26" s="4" t="s">
         <v>302</v>
       </c>
       <c r="P26" s="4" t="s">
+        <v>422</v>
+      </c>
+      <c r="Q26" s="4" t="s">
         <v>423</v>
       </c>
-      <c r="Q26" s="4" t="s">
-        <v>424</v>
-      </c>
       <c r="R26" s="4" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="S26" s="4" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
     </row>
     <row r="27" spans="1:19" ht="58" x14ac:dyDescent="0.35">
@@ -3256,7 +3255,7 @@
         <v>26</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C27" s="4" t="s">
         <v>41</v>
@@ -3291,7 +3290,7 @@
         <v>27</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C28" s="4" t="s">
         <v>42</v>
@@ -3326,7 +3325,7 @@
         <v>28</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C29" s="4" t="s">
         <v>43</v>
@@ -3364,7 +3363,7 @@
         <v>29</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C30" s="4" t="s">
         <v>44</v>
@@ -3396,7 +3395,7 @@
         <v>30</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C31" s="4" t="s">
         <v>45</v>
@@ -3407,8 +3406,8 @@
       <c r="E31" s="1" t="s">
         <v>242</v>
       </c>
-      <c r="F31" s="4" t="s">
-        <v>403</v>
+      <c r="F31" s="14" t="s">
+        <v>252</v>
       </c>
       <c r="G31" s="4" t="s">
         <v>312</v>
@@ -3437,7 +3436,7 @@
         <v>31</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C32" s="4" t="s">
         <v>46</v>
@@ -3469,7 +3468,7 @@
         <v>32</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C33" s="4" t="s">
         <v>47</v>
@@ -3499,10 +3498,10 @@
         <v>317</v>
       </c>
       <c r="O33" s="4" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="P33" s="4" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
     </row>
     <row r="34" spans="1:21" x14ac:dyDescent="0.35">
@@ -3510,7 +3509,7 @@
         <v>33</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C34" s="4" t="s">
         <v>48</v>
@@ -3542,7 +3541,7 @@
         <v>34</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C35" s="4" t="s">
         <v>49</v>
@@ -3574,7 +3573,7 @@
         <v>35</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C36" s="4" t="s">
         <v>50</v>
@@ -3606,7 +3605,7 @@
         <v>36</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C37" s="4" t="s">
         <v>51</v>
@@ -3638,7 +3637,7 @@
         <v>37</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C38" s="4" t="s">
         <v>52</v>
@@ -3670,7 +3669,7 @@
         <v>38</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C39" s="4" t="s">
         <v>53</v>
@@ -3702,7 +3701,7 @@
         <v>39</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C40" s="4" t="s">
         <v>54</v>
@@ -3732,19 +3731,19 @@
         <v>357</v>
       </c>
       <c r="Q40" s="4" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="R40" s="4" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="S40" s="4" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="T40" s="4" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="U40" s="4" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
     </row>
     <row r="41" spans="1:21" ht="43.5" x14ac:dyDescent="0.35">
@@ -3752,7 +3751,7 @@
         <v>40</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C41" s="4" t="s">
         <v>55</v>
@@ -3787,7 +3786,7 @@
         <v>41</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C42" s="4" t="s">
         <v>56</v>
@@ -3817,19 +3816,19 @@
         <v>358</v>
       </c>
       <c r="Q42" s="4" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="R42" s="4" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="S42" s="4" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="T42" s="4" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="U42" s="4" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
     </row>
     <row r="43" spans="1:21" ht="43.5" x14ac:dyDescent="0.35">
@@ -3837,7 +3836,7 @@
         <v>42</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C43" s="4" t="s">
         <v>57</v>
@@ -3872,7 +3871,7 @@
         <v>43</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C44" s="4" t="s">
         <v>58</v>
@@ -3899,19 +3898,19 @@
         <v>275</v>
       </c>
       <c r="Q44" s="4" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="R44" s="4" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="S44" s="4" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="T44" s="4" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="U44" s="4" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
     </row>
     <row r="45" spans="1:21" ht="362.5" x14ac:dyDescent="0.35">
@@ -3919,7 +3918,7 @@
         <v>44</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C45" s="4" t="s">
         <v>59</v>
@@ -3952,7 +3951,7 @@
         <v>320</v>
       </c>
       <c r="N45" s="4" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="P45" s="4" t="s">
         <v>386</v>
@@ -3963,7 +3962,7 @@
         <v>45</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C46" s="4" t="s">
         <v>60</v>
@@ -3999,7 +3998,7 @@
         <v>327</v>
       </c>
       <c r="P46" s="4" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
     </row>
     <row r="47" spans="1:21" ht="43.5" x14ac:dyDescent="0.35">
@@ -4007,7 +4006,7 @@
         <v>46</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C47" s="4" t="s">
         <v>61</v>
@@ -4051,7 +4050,7 @@
         <v>47</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C48" s="4" t="s">
         <v>62</v>
@@ -4063,7 +4062,7 @@
         <v>242</v>
       </c>
       <c r="F48" s="4" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="G48" s="4" t="s">
         <v>334</v>
@@ -4095,7 +4094,7 @@
         <v>48</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C49" s="4" t="s">
         <v>63</v>
@@ -4107,7 +4106,7 @@
         <v>244</v>
       </c>
       <c r="F49" s="4" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="G49" s="4" t="s">
         <v>337</v>
@@ -4125,7 +4124,7 @@
         <v>265</v>
       </c>
       <c r="N49" s="4" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="P49" s="4" t="s">
         <v>389</v>
@@ -4136,7 +4135,7 @@
         <v>49</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C50" s="4" t="s">
         <v>64</v>
@@ -4174,7 +4173,7 @@
         <v>50</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C51" s="4" t="s">
         <v>65</v>
@@ -4201,10 +4200,10 @@
         <v>265</v>
       </c>
       <c r="N51" s="4" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="P51" s="4" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
     </row>
     <row r="52" spans="1:16" ht="29" x14ac:dyDescent="0.35">
@@ -4212,7 +4211,7 @@
         <v>51</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C52" s="4" t="s">
         <v>66</v>
@@ -4227,7 +4226,7 @@
         <v>252</v>
       </c>
       <c r="J52" s="4" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="K52" s="1" t="s">
         <v>275</v>
@@ -4242,7 +4241,7 @@
         <v>275</v>
       </c>
       <c r="P52" s="4" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="53" spans="1:16" ht="29" x14ac:dyDescent="0.35">
@@ -4250,7 +4249,7 @@
         <v>52</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C53" s="4" t="s">
         <v>67</v>
@@ -4282,7 +4281,7 @@
         <v>53</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C54" s="4" t="s">
         <v>68</v>
@@ -4314,7 +4313,7 @@
         <v>54</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C55" s="4" t="s">
         <v>69</v>
@@ -4346,7 +4345,7 @@
         <v>55</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C56" s="4" t="s">
         <v>70</v>
@@ -4378,7 +4377,7 @@
         <v>56</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C57" s="4" t="s">
         <v>71</v>
@@ -4410,7 +4409,7 @@
         <v>57</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C58" s="4" t="s">
         <v>72</v>
@@ -4442,7 +4441,7 @@
         <v>58</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C59" s="4" t="s">
         <v>73</v>
@@ -4474,7 +4473,7 @@
         <v>59</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C60" s="4" t="s">
         <v>74</v>
@@ -4506,7 +4505,7 @@
         <v>60</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C61" s="4" t="s">
         <v>75</v>
@@ -4538,7 +4537,7 @@
         <v>61</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C62" s="4" t="s">
         <v>76</v>
@@ -4570,7 +4569,7 @@
         <v>62</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C63" s="4" t="s">
         <v>77</v>
@@ -4602,7 +4601,7 @@
         <v>63</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C64" s="4" t="s">
         <v>78</v>
@@ -4634,7 +4633,7 @@
         <v>64</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C65" s="4" t="s">
         <v>79</v>
@@ -4666,7 +4665,7 @@
         <v>65</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C66" s="4" t="s">
         <v>80</v>
@@ -4698,7 +4697,7 @@
         <v>66</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C67" s="4" t="s">
         <v>81</v>
@@ -4730,7 +4729,7 @@
         <v>67</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C68" s="4" t="s">
         <v>82</v>
@@ -4763,10 +4762,10 @@
         <v>317</v>
       </c>
       <c r="O68" s="5" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="P68" s="4" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="69" spans="1:17" ht="72.5" x14ac:dyDescent="0.35">
@@ -4774,7 +4773,7 @@
         <v>68</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C69" s="4" t="s">
         <v>83</v>
@@ -4819,7 +4818,7 @@
         <v>69</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C70" s="4" t="s">
         <v>84</v>
@@ -4851,7 +4850,7 @@
         <v>70</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C71" s="4" t="s">
         <v>85</v>
@@ -4883,7 +4882,7 @@
         <v>71</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C72" s="4" t="s">
         <v>86</v>
@@ -4921,7 +4920,7 @@
         <v>72</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C73" s="4" t="s">
         <v>87</v>
@@ -4959,7 +4958,7 @@
         <v>73</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C74" s="4" t="s">
         <v>88</v>
@@ -4991,7 +4990,7 @@
         <v>74</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C75" s="4" t="s">
         <v>89</v>
@@ -5023,7 +5022,7 @@
         <v>75</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C76" s="4" t="s">
         <v>90</v>
@@ -5061,7 +5060,7 @@
         <v>76</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C77" s="4" t="s">
         <v>91</v>
@@ -5097,7 +5096,7 @@
         <v>391</v>
       </c>
       <c r="P77" s="4" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="78" spans="1:17" ht="101.5" x14ac:dyDescent="0.35">
@@ -5105,7 +5104,7 @@
         <v>77</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C78" s="4" t="s">
         <v>92</v>
@@ -5126,7 +5125,7 @@
         <v>346</v>
       </c>
       <c r="J78" s="4" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="K78" s="1" t="s">
         <v>249</v>
@@ -5138,13 +5137,13 @@
         <v>265</v>
       </c>
       <c r="N78" s="4" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="O78" s="4" t="s">
+        <v>438</v>
+      </c>
+      <c r="P78" s="4" t="s">
         <v>439</v>
-      </c>
-      <c r="P78" s="4" t="s">
-        <v>440</v>
       </c>
       <c r="Q78" s="5"/>
     </row>
@@ -5153,7 +5152,7 @@
         <v>78</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C79" s="4" t="s">
         <v>93</v>
@@ -5174,7 +5173,7 @@
         <v>346</v>
       </c>
       <c r="J79" s="4" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="K79" s="1" t="s">
         <v>249</v>
@@ -5189,7 +5188,7 @@
         <v>272</v>
       </c>
       <c r="P79" s="4" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="80" spans="1:17" x14ac:dyDescent="0.35">
@@ -5197,7 +5196,7 @@
         <v>79</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C80" s="4" t="s">
         <v>94</v>
@@ -5229,7 +5228,7 @@
         <v>80</v>
       </c>
       <c r="B81" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C81" s="4" t="s">
         <v>95</v>
@@ -5267,7 +5266,7 @@
         <v>81</v>
       </c>
       <c r="B82" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C82" s="4" t="s">
         <v>96</v>
@@ -5285,7 +5284,7 @@
         <v>365</v>
       </c>
       <c r="J82" s="4" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="K82" s="1" t="s">
         <v>249</v>
@@ -5297,22 +5296,22 @@
         <v>265</v>
       </c>
       <c r="N82" s="4" t="s">
+        <v>461</v>
+      </c>
+      <c r="O82" s="4" t="s">
+        <v>409</v>
+      </c>
+      <c r="P82" s="4" t="s">
         <v>462</v>
       </c>
-      <c r="O82" s="4" t="s">
-        <v>410</v>
-      </c>
-      <c r="P82" s="4" t="s">
-        <v>463</v>
-      </c>
       <c r="Q82" s="5" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="R82" s="4" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="S82" s="4" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
     <row r="83" spans="1:19" ht="159.5" x14ac:dyDescent="0.35">
@@ -5320,7 +5319,7 @@
         <v>82</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C83" s="4" t="s">
         <v>97</v>
@@ -5338,7 +5337,7 @@
         <v>365</v>
       </c>
       <c r="J83" s="4" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="K83" s="1" t="s">
         <v>249</v>
@@ -5350,22 +5349,22 @@
         <v>265</v>
       </c>
       <c r="N83" s="4" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="O83" s="4" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="P83" s="4" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="Q83" s="5" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="R83" s="4" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="S83" s="4" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
     <row r="84" spans="1:19" ht="159.5" x14ac:dyDescent="0.35">
@@ -5373,7 +5372,7 @@
         <v>83</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C84" s="4" t="s">
         <v>98</v>
@@ -5391,7 +5390,7 @@
         <v>365</v>
       </c>
       <c r="J84" s="4" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="K84" s="1" t="s">
         <v>249</v>
@@ -5403,22 +5402,22 @@
         <v>265</v>
       </c>
       <c r="N84" s="4" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="O84" s="4" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="P84" s="4" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="Q84" s="5" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="R84" s="4" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="S84" s="4" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
     <row r="85" spans="1:19" ht="159.5" x14ac:dyDescent="0.35">
@@ -5426,7 +5425,7 @@
         <v>84</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C85" s="4" t="s">
         <v>99</v>
@@ -5444,7 +5443,7 @@
         <v>365</v>
       </c>
       <c r="J85" s="4" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="K85" s="1" t="s">
         <v>249</v>
@@ -5456,22 +5455,22 @@
         <v>265</v>
       </c>
       <c r="N85" s="4" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="O85" s="4" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="P85" s="4" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="Q85" s="5" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="R85" s="4" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="S85" s="4" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
     <row r="86" spans="1:19" ht="159.5" x14ac:dyDescent="0.35">
@@ -5479,7 +5478,7 @@
         <v>85</v>
       </c>
       <c r="B86" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C86" s="4" t="s">
         <v>100</v>
@@ -5497,7 +5496,7 @@
         <v>365</v>
       </c>
       <c r="J86" s="4" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="K86" s="1" t="s">
         <v>249</v>
@@ -5509,22 +5508,22 @@
         <v>265</v>
       </c>
       <c r="N86" s="4" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="O86" s="4" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="P86" s="4" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="Q86" s="5" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="R86" s="4" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="S86" s="4" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
     <row r="87" spans="1:19" ht="159.5" x14ac:dyDescent="0.35">
@@ -5532,7 +5531,7 @@
         <v>86</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C87" s="4" t="s">
         <v>101</v>
@@ -5550,7 +5549,7 @@
         <v>365</v>
       </c>
       <c r="J87" s="4" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="K87" s="1" t="s">
         <v>249</v>
@@ -5562,22 +5561,22 @@
         <v>265</v>
       </c>
       <c r="N87" s="4" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="O87" s="4" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="P87" s="4" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="Q87" s="5" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="R87" s="4" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="S87" s="4" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
     <row r="88" spans="1:19" ht="159.5" x14ac:dyDescent="0.35">
@@ -5585,7 +5584,7 @@
         <v>87</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C88" s="4" t="s">
         <v>102</v>
@@ -5603,7 +5602,7 @@
         <v>365</v>
       </c>
       <c r="J88" s="4" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="K88" s="1" t="s">
         <v>249</v>
@@ -5615,22 +5614,22 @@
         <v>265</v>
       </c>
       <c r="N88" s="4" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="O88" s="4" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="P88" s="4" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="Q88" s="5" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="R88" s="4" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="S88" s="4" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
     <row r="89" spans="1:19" ht="159.5" x14ac:dyDescent="0.35">
@@ -5638,7 +5637,7 @@
         <v>88</v>
       </c>
       <c r="B89" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C89" s="4" t="s">
         <v>103</v>
@@ -5656,7 +5655,7 @@
         <v>365</v>
       </c>
       <c r="J89" s="4" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="K89" s="1" t="s">
         <v>249</v>
@@ -5668,22 +5667,22 @@
         <v>265</v>
       </c>
       <c r="N89" s="4" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="O89" s="4" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="P89" s="4" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="Q89" s="5" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="R89" s="4" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="S89" s="4" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
     <row r="90" spans="1:19" ht="159.5" x14ac:dyDescent="0.35">
@@ -5691,7 +5690,7 @@
         <v>89</v>
       </c>
       <c r="B90" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C90" s="4" t="s">
         <v>104</v>
@@ -5709,7 +5708,7 @@
         <v>365</v>
       </c>
       <c r="J90" s="4" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="K90" s="1" t="s">
         <v>249</v>
@@ -5721,22 +5720,22 @@
         <v>265</v>
       </c>
       <c r="N90" s="4" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="O90" s="4" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="P90" s="4" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="Q90" s="5" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="R90" s="4" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="S90" s="4" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
     <row r="91" spans="1:19" ht="159.5" x14ac:dyDescent="0.35">
@@ -5744,7 +5743,7 @@
         <v>90</v>
       </c>
       <c r="B91" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C91" s="4" t="s">
         <v>105</v>
@@ -5762,7 +5761,7 @@
         <v>365</v>
       </c>
       <c r="J91" s="4" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="K91" s="1" t="s">
         <v>249</v>
@@ -5774,22 +5773,22 @@
         <v>265</v>
       </c>
       <c r="N91" s="4" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="O91" s="4" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="P91" s="4" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="Q91" s="5" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="R91" s="13" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="S91" s="4" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
     <row r="92" spans="1:19" ht="159.5" x14ac:dyDescent="0.35">
@@ -5797,7 +5796,7 @@
         <v>91</v>
       </c>
       <c r="B92" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C92" s="4" t="s">
         <v>106</v>
@@ -5815,7 +5814,7 @@
         <v>365</v>
       </c>
       <c r="J92" s="4" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="K92" s="1" t="s">
         <v>249</v>
@@ -5827,22 +5826,22 @@
         <v>265</v>
       </c>
       <c r="N92" s="4" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="O92" s="4" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="P92" s="4" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="Q92" s="5" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="R92" s="13" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="S92" s="4" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
     <row r="93" spans="1:19" ht="159.5" x14ac:dyDescent="0.35">
@@ -5850,7 +5849,7 @@
         <v>92</v>
       </c>
       <c r="B93" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C93" s="4" t="s">
         <v>107</v>
@@ -5868,7 +5867,7 @@
         <v>365</v>
       </c>
       <c r="J93" s="4" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="K93" s="1" t="s">
         <v>249</v>
@@ -5880,22 +5879,22 @@
         <v>265</v>
       </c>
       <c r="N93" s="4" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="O93" s="4" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="P93" s="4" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="Q93" s="5" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="R93" s="13" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="S93" s="4" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
     <row r="94" spans="1:19" ht="159.5" x14ac:dyDescent="0.35">
@@ -5903,7 +5902,7 @@
         <v>93</v>
       </c>
       <c r="B94" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C94" s="4" t="s">
         <v>108</v>
@@ -5921,7 +5920,7 @@
         <v>365</v>
       </c>
       <c r="J94" s="4" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="K94" s="1" t="s">
         <v>249</v>
@@ -5933,22 +5932,22 @@
         <v>265</v>
       </c>
       <c r="N94" s="4" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="O94" s="4" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="P94" s="4" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="Q94" s="5" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="R94" s="13" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="S94" s="4" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
     <row r="95" spans="1:19" ht="159.5" x14ac:dyDescent="0.35">
@@ -5956,7 +5955,7 @@
         <v>94</v>
       </c>
       <c r="B95" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C95" s="4" t="s">
         <v>109</v>
@@ -5974,7 +5973,7 @@
         <v>365</v>
       </c>
       <c r="J95" s="4" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="K95" s="1" t="s">
         <v>249</v>
@@ -5986,22 +5985,22 @@
         <v>265</v>
       </c>
       <c r="N95" s="4" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="O95" s="4" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="P95" s="4" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="Q95" s="5" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="R95" s="13" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="S95" s="4" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
     <row r="96" spans="1:19" ht="159.5" x14ac:dyDescent="0.35">
@@ -6009,7 +6008,7 @@
         <v>95</v>
       </c>
       <c r="B96" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C96" s="4" t="s">
         <v>110</v>
@@ -6027,7 +6026,7 @@
         <v>365</v>
       </c>
       <c r="J96" s="4" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="K96" s="1" t="s">
         <v>249</v>
@@ -6039,22 +6038,22 @@
         <v>265</v>
       </c>
       <c r="N96" s="4" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="O96" s="4" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="P96" s="4" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="Q96" s="5" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="R96" s="13" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="S96" s="4" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
     <row r="97" spans="1:19" ht="159.5" x14ac:dyDescent="0.35">
@@ -6062,7 +6061,7 @@
         <v>96</v>
       </c>
       <c r="B97" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C97" s="4" t="s">
         <v>111</v>
@@ -6080,7 +6079,7 @@
         <v>365</v>
       </c>
       <c r="J97" s="4" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="K97" s="1" t="s">
         <v>249</v>
@@ -6092,22 +6091,22 @@
         <v>265</v>
       </c>
       <c r="N97" s="4" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="O97" s="4" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="P97" s="4" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="Q97" s="5" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="R97" s="13" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="S97" s="4" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
     <row r="98" spans="1:19" ht="159.5" x14ac:dyDescent="0.35">
@@ -6115,7 +6114,7 @@
         <v>97</v>
       </c>
       <c r="B98" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C98" s="4" t="s">
         <v>112</v>
@@ -6133,7 +6132,7 @@
         <v>365</v>
       </c>
       <c r="J98" s="4" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="K98" s="1" t="s">
         <v>249</v>
@@ -6145,22 +6144,22 @@
         <v>265</v>
       </c>
       <c r="N98" s="4" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="O98" s="4" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="P98" s="4" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="Q98" s="5" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="R98" s="13" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="S98" s="4" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
     <row r="99" spans="1:19" ht="159.5" x14ac:dyDescent="0.35">
@@ -6168,7 +6167,7 @@
         <v>98</v>
       </c>
       <c r="B99" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C99" s="4" t="s">
         <v>113</v>
@@ -6186,7 +6185,7 @@
         <v>365</v>
       </c>
       <c r="J99" s="4" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="K99" s="1" t="s">
         <v>249</v>
@@ -6198,22 +6197,22 @@
         <v>265</v>
       </c>
       <c r="N99" s="4" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="O99" s="4" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="P99" s="4" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="Q99" s="5" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="R99" s="13" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="S99" s="4" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
     <row r="100" spans="1:19" ht="159.5" x14ac:dyDescent="0.35">
@@ -6221,7 +6220,7 @@
         <v>99</v>
       </c>
       <c r="B100" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C100" s="4" t="s">
         <v>114</v>
@@ -6239,7 +6238,7 @@
         <v>365</v>
       </c>
       <c r="J100" s="4" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="K100" s="1" t="s">
         <v>249</v>
@@ -6251,22 +6250,22 @@
         <v>265</v>
       </c>
       <c r="N100" s="4" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="O100" s="4" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="P100" s="4" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="Q100" s="5" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="R100" s="13" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="S100" s="4" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
     <row r="101" spans="1:19" ht="58" x14ac:dyDescent="0.35">
@@ -6274,7 +6273,7 @@
         <v>100</v>
       </c>
       <c r="B101" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C101" s="4" t="s">
         <v>115</v>
@@ -6295,7 +6294,7 @@
         <v>346</v>
       </c>
       <c r="J101" s="4" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="K101" s="1" t="s">
         <v>249</v>
@@ -6315,7 +6314,7 @@
         <v>101</v>
       </c>
       <c r="B102" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C102" s="4" t="s">
         <v>116</v>
@@ -6347,7 +6346,7 @@
         <v>102</v>
       </c>
       <c r="B103" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C103" s="4" t="s">
         <v>117</v>
@@ -6379,7 +6378,7 @@
         <v>103</v>
       </c>
       <c r="B104" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C104" s="4" t="s">
         <v>118</v>
@@ -6400,7 +6399,7 @@
         <v>370</v>
       </c>
       <c r="J104" s="4" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="K104" s="1" t="s">
         <v>249</v>
@@ -6420,7 +6419,7 @@
         <v>104</v>
       </c>
       <c r="B105" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C105" s="4" t="s">
         <v>119</v>
@@ -6438,7 +6437,7 @@
         <v>375</v>
       </c>
       <c r="J105" s="4" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="K105" s="1" t="s">
         <v>249</v>
@@ -6458,7 +6457,7 @@
         <v>105</v>
       </c>
       <c r="B106" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C106" s="4" t="s">
         <v>120</v>
@@ -6479,7 +6478,7 @@
         <v>370</v>
       </c>
       <c r="J106" s="4" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="K106" s="1" t="s">
         <v>249</v>
@@ -6499,7 +6498,7 @@
         <v>106</v>
       </c>
       <c r="B107" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C107" s="4" t="s">
         <v>121</v>
@@ -6531,7 +6530,7 @@
         <v>107</v>
       </c>
       <c r="B108" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C108" s="4" t="s">
         <v>122</v>
@@ -6563,7 +6562,7 @@
         <v>108</v>
       </c>
       <c r="B109" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C109" s="4" t="s">
         <v>123</v>
@@ -6595,7 +6594,7 @@
         <v>109</v>
       </c>
       <c r="B110" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C110" s="4" t="s">
         <v>124</v>
@@ -6627,7 +6626,7 @@
         <v>110</v>
       </c>
       <c r="B111" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C111" s="4" t="s">
         <v>125</v>
@@ -6668,7 +6667,7 @@
         <v>111</v>
       </c>
       <c r="B112" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C112" s="4" t="s">
         <v>126</v>
@@ -6700,7 +6699,7 @@
         <v>112</v>
       </c>
       <c r="B113" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C113" s="4" t="s">
         <v>127</v>

</xml_diff>

<commit_message>
use gsk_id as id
</commit_message>
<xml_diff>
--- a/longitudinal/data_processing_elements_longitudinal-MSC.xlsx
+++ b/longitudinal/data_processing_elements_longitudinal-MSC.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Computer\twey working files\ProPASS\MSC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96E93E5B-C4F7-4FEA-AF72-30623FD5EC2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09CD1780-27BB-49F4-A248-B5028C6D4359}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{EBFE0AAE-9F6E-4351-BDB4-692162CD990C}"/>
   </bookViews>
@@ -831,9 +831,6 @@
 ELSE=NA)</t>
   </si>
   <si>
-    <t>patient_key</t>
-  </si>
-  <si>
     <t>Participant ID</t>
   </si>
   <si>
@@ -1679,6 +1676,9 @@
   </si>
   <si>
     <t>Study variable is based on having "Diabetes or Blood Sugar". Study confirmed that this is self-reported diabetes.</t>
+  </si>
+  <si>
+    <t>gsk_id</t>
   </si>
 </sst>
 </file>
@@ -2176,10 +2176,10 @@
         <v>0</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="D1" s="8" t="s">
         <v>128</v>
@@ -2200,10 +2200,10 @@
         <v>5</v>
       </c>
       <c r="J1" s="10" t="s">
+        <v>395</v>
+      </c>
+      <c r="K1" s="10" t="s">
         <v>396</v>
-      </c>
-      <c r="K1" s="10" t="s">
-        <v>397</v>
       </c>
       <c r="L1" s="11" t="s">
         <v>6</v>
@@ -2241,7 +2241,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>16</v>
@@ -2252,11 +2252,11 @@
       <c r="E2" s="1" t="s">
         <v>241</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="7" t="s">
+        <v>466</v>
+      </c>
+      <c r="G2" s="1" t="s">
         <v>261</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>262</v>
       </c>
       <c r="K2" s="1" t="s">
         <v>249</v>
@@ -2267,8 +2267,8 @@
       <c r="M2" s="1" t="s">
         <v>251</v>
       </c>
-      <c r="N2" s="1" t="s">
-        <v>261</v>
+      <c r="N2" s="7" t="s">
+        <v>466</v>
       </c>
     </row>
     <row r="3" spans="1:21" x14ac:dyDescent="0.35">
@@ -2276,7 +2276,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>17</v>
@@ -2300,7 +2300,7 @@
         <v>253</v>
       </c>
       <c r="N3" s="1" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="Q3" s="5"/>
     </row>
@@ -2309,7 +2309,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>18</v>
@@ -2333,10 +2333,10 @@
         <v>253</v>
       </c>
       <c r="N4" s="1" t="s">
+        <v>409</v>
+      </c>
+      <c r="P4" s="4" t="s">
         <v>410</v>
-      </c>
-      <c r="P4" s="4" t="s">
-        <v>411</v>
       </c>
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.35">
@@ -2344,7 +2344,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>19</v>
@@ -2368,7 +2368,7 @@
         <v>253</v>
       </c>
       <c r="N5" s="1" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="6" spans="1:21" ht="58" x14ac:dyDescent="0.35">
@@ -2376,7 +2376,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>20</v>
@@ -2403,25 +2403,25 @@
         <v>255</v>
       </c>
       <c r="N6" s="7" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="O6" s="4" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="Q6" s="4" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="R6" s="4" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="S6" s="4" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="T6" s="4" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="U6" s="4" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
     </row>
     <row r="7" spans="1:21" ht="58" x14ac:dyDescent="0.35">
@@ -2429,7 +2429,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>21</v>
@@ -2467,7 +2467,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>22</v>
@@ -2479,7 +2479,7 @@
         <v>242</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="G8" s="1" t="s">
         <v>135</v>
@@ -2491,16 +2491,16 @@
         <v>249</v>
       </c>
       <c r="L8" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="M8" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="M8" s="1" t="s">
+      <c r="N8" s="4" t="s">
+        <v>398</v>
+      </c>
+      <c r="O8" s="4" t="s">
         <v>265</v>
-      </c>
-      <c r="N8" s="4" t="s">
-        <v>399</v>
-      </c>
-      <c r="O8" s="4" t="s">
-        <v>266</v>
       </c>
     </row>
     <row r="9" spans="1:21" ht="188.5" x14ac:dyDescent="0.35">
@@ -2508,7 +2508,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>23</v>
@@ -2520,34 +2520,34 @@
         <v>242</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="G9" s="1" t="s">
         <v>136</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="K9" s="1" t="s">
         <v>249</v>
       </c>
       <c r="L9" s="1" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="M9" s="1" t="s">
         <v>259</v>
       </c>
       <c r="N9" s="4" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="Q9" s="4" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="R9" s="4" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="S9" s="4" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
     </row>
     <row r="10" spans="1:21" ht="188.5" x14ac:dyDescent="0.35">
@@ -2555,7 +2555,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>24</v>
@@ -2567,25 +2567,25 @@
         <v>242</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="G10" s="1" t="s">
         <v>136</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="K10" s="1" t="s">
         <v>249</v>
       </c>
       <c r="L10" s="1" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="M10" s="1" t="s">
         <v>259</v>
       </c>
       <c r="N10" s="4" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="11" spans="1:21" ht="58" x14ac:dyDescent="0.35">
@@ -2593,7 +2593,7 @@
         <v>10</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>25</v>
@@ -2605,13 +2605,13 @@
         <v>242</v>
       </c>
       <c r="F11" s="1" t="s">
+        <v>268</v>
+      </c>
+      <c r="G11" s="1" t="s">
         <v>269</v>
       </c>
-      <c r="G11" s="1" t="s">
+      <c r="H11" s="4" t="s">
         <v>270</v>
-      </c>
-      <c r="H11" s="4" t="s">
-        <v>271</v>
       </c>
       <c r="K11" s="1" t="s">
         <v>249</v>
@@ -2623,7 +2623,7 @@
         <v>259</v>
       </c>
       <c r="N11" s="4" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="12" spans="1:21" ht="58" x14ac:dyDescent="0.35">
@@ -2631,7 +2631,7 @@
         <v>11</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>26</v>
@@ -2643,13 +2643,13 @@
         <v>242</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="G12" s="1" t="s">
+        <v>272</v>
+      </c>
+      <c r="H12" s="4" t="s">
         <v>273</v>
-      </c>
-      <c r="H12" s="4" t="s">
-        <v>274</v>
       </c>
       <c r="K12" s="1" t="s">
         <v>249</v>
@@ -2664,7 +2664,7 @@
         <v>260</v>
       </c>
       <c r="O12" s="4" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="13" spans="1:21" ht="43.5" x14ac:dyDescent="0.35">
@@ -2672,7 +2672,7 @@
         <v>12</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>27</v>
@@ -2687,16 +2687,16 @@
         <v>252</v>
       </c>
       <c r="K13" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="L13" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="L13" s="1" t="s">
-        <v>276</v>
-      </c>
       <c r="M13" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="N13" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="14" spans="1:21" ht="174" x14ac:dyDescent="0.35">
@@ -2704,7 +2704,7 @@
         <v>13</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>28</v>
@@ -2716,25 +2716,25 @@
         <v>241</v>
       </c>
       <c r="F14" s="4" t="s">
+        <v>380</v>
+      </c>
+      <c r="G14" s="4" t="s">
         <v>381</v>
       </c>
-      <c r="G14" s="4" t="s">
-        <v>382</v>
-      </c>
       <c r="H14" s="4" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="K14" s="1" t="s">
         <v>249</v>
       </c>
       <c r="L14" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="M14" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="M14" s="1" t="s">
-        <v>265</v>
-      </c>
       <c r="N14" s="4" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="15" spans="1:21" ht="58" x14ac:dyDescent="0.35">
@@ -2742,7 +2742,7 @@
         <v>14</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C15" s="4" t="s">
         <v>29</v>
@@ -2754,28 +2754,28 @@
         <v>242</v>
       </c>
       <c r="F15" s="1" t="s">
+        <v>268</v>
+      </c>
+      <c r="G15" s="1" t="s">
         <v>269</v>
       </c>
-      <c r="G15" s="1" t="s">
+      <c r="H15" s="4" t="s">
         <v>270</v>
-      </c>
-      <c r="H15" s="4" t="s">
-        <v>271</v>
       </c>
       <c r="K15" s="1" t="s">
         <v>249</v>
       </c>
       <c r="L15" s="1" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="M15" s="1" t="s">
         <v>259</v>
       </c>
       <c r="N15" s="4" t="s">
+        <v>413</v>
+      </c>
+      <c r="P15" s="4" t="s">
         <v>414</v>
-      </c>
-      <c r="P15" s="4" t="s">
-        <v>415</v>
       </c>
     </row>
     <row r="16" spans="1:21" ht="116" x14ac:dyDescent="0.35">
@@ -2783,7 +2783,7 @@
         <v>15</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>30</v>
@@ -2795,25 +2795,25 @@
         <v>242</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="G16" s="1" t="s">
         <v>143</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="K16" s="1" t="s">
         <v>249</v>
       </c>
       <c r="L16" s="1" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="M16" s="1" t="s">
         <v>259</v>
       </c>
       <c r="N16" s="4" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="17" spans="1:19" ht="87" x14ac:dyDescent="0.35">
@@ -2821,7 +2821,7 @@
         <v>16</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C17" s="4" t="s">
         <v>31</v>
@@ -2836,7 +2836,7 @@
         <v>252</v>
       </c>
       <c r="J17" s="4" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="K17" s="1" t="s">
         <v>249</v>
@@ -2848,10 +2848,10 @@
         <v>253</v>
       </c>
       <c r="N17" s="1" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="P17" s="4" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
     </row>
     <row r="18" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
@@ -2859,7 +2859,7 @@
         <v>17</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C18" s="4" t="s">
         <v>32</v>
@@ -2871,10 +2871,10 @@
         <v>244</v>
       </c>
       <c r="F18" s="1" t="s">
+        <v>281</v>
+      </c>
+      <c r="G18" s="1" t="s">
         <v>282</v>
-      </c>
-      <c r="G18" s="1" t="s">
-        <v>283</v>
       </c>
       <c r="I18" s="4" t="s">
         <v>246</v>
@@ -2886,10 +2886,10 @@
         <v>250</v>
       </c>
       <c r="M18" s="1" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="N18" s="4" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
     <row r="19" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
@@ -2897,7 +2897,7 @@
         <v>18</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>33</v>
@@ -2909,10 +2909,10 @@
         <v>242</v>
       </c>
       <c r="F19" s="1" t="s">
+        <v>281</v>
+      </c>
+      <c r="G19" s="1" t="s">
         <v>282</v>
-      </c>
-      <c r="G19" s="1" t="s">
-        <v>283</v>
       </c>
       <c r="I19" s="4" t="s">
         <v>246</v>
@@ -2921,25 +2921,25 @@
         <v>249</v>
       </c>
       <c r="L19" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="M19" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="M19" s="1" t="s">
-        <v>265</v>
-      </c>
       <c r="N19" s="4" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="O19" s="4" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="Q19" s="4" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="R19" s="4" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="S19" s="4" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
     </row>
     <row r="20" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
@@ -2947,7 +2947,7 @@
         <v>19</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C20" s="4" t="s">
         <v>34</v>
@@ -2959,10 +2959,10 @@
         <v>244</v>
       </c>
       <c r="F20" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="G20" s="1" t="s">
         <v>286</v>
-      </c>
-      <c r="G20" s="1" t="s">
-        <v>287</v>
       </c>
       <c r="I20" s="4" t="s">
         <v>247</v>
@@ -2974,10 +2974,10 @@
         <v>250</v>
       </c>
       <c r="M20" s="1" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="N20" s="4" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="21" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
@@ -2985,7 +2985,7 @@
         <v>20</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C21" s="4" t="s">
         <v>35</v>
@@ -2997,10 +2997,10 @@
         <v>242</v>
       </c>
       <c r="F21" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="G21" s="1" t="s">
         <v>286</v>
-      </c>
-      <c r="G21" s="1" t="s">
-        <v>287</v>
       </c>
       <c r="I21" s="4" t="s">
         <v>247</v>
@@ -3009,25 +3009,25 @@
         <v>249</v>
       </c>
       <c r="L21" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="M21" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="M21" s="1" t="s">
-        <v>265</v>
-      </c>
       <c r="N21" s="4" t="s">
+        <v>288</v>
+      </c>
+      <c r="O21" s="4" t="s">
         <v>289</v>
       </c>
-      <c r="O21" s="4" t="s">
-        <v>290</v>
-      </c>
       <c r="Q21" s="4" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="R21" s="4" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="S21" s="4" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
     </row>
     <row r="22" spans="1:19" ht="58" x14ac:dyDescent="0.35">
@@ -3035,7 +3035,7 @@
         <v>21</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C22" s="4" t="s">
         <v>36</v>
@@ -3047,28 +3047,28 @@
         <v>244</v>
       </c>
       <c r="F22" s="4" t="s">
+        <v>290</v>
+      </c>
+      <c r="G22" s="4" t="s">
         <v>291</v>
       </c>
-      <c r="G22" s="4" t="s">
+      <c r="I22" s="4" t="s">
         <v>292</v>
-      </c>
-      <c r="I22" s="4" t="s">
-        <v>293</v>
       </c>
       <c r="K22" s="1" t="s">
         <v>249</v>
       </c>
       <c r="L22" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="M22" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="M22" s="1" t="s">
-        <v>265</v>
-      </c>
       <c r="N22" s="4" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="O22" s="4" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
     </row>
     <row r="23" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
@@ -3076,7 +3076,7 @@
         <v>22</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C23" s="4" t="s">
         <v>37</v>
@@ -3088,10 +3088,10 @@
         <v>244</v>
       </c>
       <c r="F23" s="1" t="s">
+        <v>294</v>
+      </c>
+      <c r="G23" s="1" t="s">
         <v>295</v>
-      </c>
-      <c r="G23" s="1" t="s">
-        <v>296</v>
       </c>
       <c r="I23" s="4" t="s">
         <v>246</v>
@@ -3103,10 +3103,10 @@
         <v>250</v>
       </c>
       <c r="M23" s="1" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="N23" s="4" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="24" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
@@ -3114,7 +3114,7 @@
         <v>23</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C24" s="4" t="s">
         <v>38</v>
@@ -3126,10 +3126,10 @@
         <v>242</v>
       </c>
       <c r="F24" s="1" t="s">
+        <v>294</v>
+      </c>
+      <c r="G24" s="1" t="s">
         <v>295</v>
-      </c>
-      <c r="G24" s="1" t="s">
-        <v>296</v>
       </c>
       <c r="I24" s="4" t="s">
         <v>246</v>
@@ -3138,25 +3138,25 @@
         <v>249</v>
       </c>
       <c r="L24" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="M24" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="M24" s="1" t="s">
-        <v>265</v>
-      </c>
       <c r="N24" s="4" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="O24" s="4" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="Q24" s="4" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="R24" s="4" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="S24" s="4" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
     </row>
     <row r="25" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
@@ -3164,7 +3164,7 @@
         <v>24</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C25" s="4" t="s">
         <v>39</v>
@@ -3176,10 +3176,10 @@
         <v>244</v>
       </c>
       <c r="F25" s="1" t="s">
+        <v>298</v>
+      </c>
+      <c r="G25" s="1" t="s">
         <v>299</v>
-      </c>
-      <c r="G25" s="1" t="s">
-        <v>300</v>
       </c>
       <c r="I25" s="4" t="s">
         <v>248</v>
@@ -3191,10 +3191,10 @@
         <v>250</v>
       </c>
       <c r="M25" s="1" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="N25" s="4" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="26" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
@@ -3202,7 +3202,7 @@
         <v>25</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C26" s="4" t="s">
         <v>40</v>
@@ -3214,10 +3214,10 @@
         <v>241</v>
       </c>
       <c r="F26" s="1" t="s">
+        <v>298</v>
+      </c>
+      <c r="G26" s="1" t="s">
         <v>299</v>
-      </c>
-      <c r="G26" s="1" t="s">
-        <v>300</v>
       </c>
       <c r="I26" s="4" t="s">
         <v>248</v>
@@ -3226,28 +3226,28 @@
         <v>249</v>
       </c>
       <c r="L26" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="M26" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="M26" s="1" t="s">
-        <v>265</v>
-      </c>
       <c r="N26" s="4" t="s">
+        <v>420</v>
+      </c>
+      <c r="O26" s="4" t="s">
+        <v>301</v>
+      </c>
+      <c r="P26" s="4" t="s">
         <v>421</v>
       </c>
-      <c r="O26" s="4" t="s">
-        <v>302</v>
-      </c>
-      <c r="P26" s="4" t="s">
+      <c r="Q26" s="4" t="s">
         <v>422</v>
       </c>
-      <c r="Q26" s="4" t="s">
-        <v>423</v>
-      </c>
       <c r="R26" s="4" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="S26" s="4" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
     </row>
     <row r="27" spans="1:19" ht="58" x14ac:dyDescent="0.35">
@@ -3255,7 +3255,7 @@
         <v>26</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C27" s="4" t="s">
         <v>41</v>
@@ -3267,10 +3267,10 @@
         <v>244</v>
       </c>
       <c r="F27" s="1" t="s">
+        <v>302</v>
+      </c>
+      <c r="G27" s="1" t="s">
         <v>303</v>
-      </c>
-      <c r="G27" s="1" t="s">
-        <v>304</v>
       </c>
       <c r="K27" s="1" t="s">
         <v>249</v>
@@ -3279,10 +3279,10 @@
         <v>250</v>
       </c>
       <c r="M27" s="1" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="N27" s="4" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="28" spans="1:19" ht="58" x14ac:dyDescent="0.35">
@@ -3290,7 +3290,7 @@
         <v>27</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C28" s="4" t="s">
         <v>42</v>
@@ -3302,10 +3302,10 @@
         <v>244</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="K28" s="1" t="s">
         <v>249</v>
@@ -3314,10 +3314,10 @@
         <v>250</v>
       </c>
       <c r="M28" s="1" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="N28" s="4" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="29" spans="1:19" ht="58" x14ac:dyDescent="0.35">
@@ -3325,7 +3325,7 @@
         <v>28</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C29" s="4" t="s">
         <v>43</v>
@@ -3337,10 +3337,10 @@
         <v>244</v>
       </c>
       <c r="F29" s="1" t="s">
+        <v>307</v>
+      </c>
+      <c r="G29" s="1" t="s">
         <v>308</v>
-      </c>
-      <c r="G29" s="1" t="s">
-        <v>309</v>
       </c>
       <c r="K29" s="1" t="s">
         <v>249</v>
@@ -3349,13 +3349,13 @@
         <v>250</v>
       </c>
       <c r="M29" s="1" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="N29" s="4" t="s">
+        <v>309</v>
+      </c>
+      <c r="O29" s="4" t="s">
         <v>310</v>
-      </c>
-      <c r="O29" s="4" t="s">
-        <v>311</v>
       </c>
     </row>
     <row r="30" spans="1:19" ht="29" x14ac:dyDescent="0.35">
@@ -3363,7 +3363,7 @@
         <v>29</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C30" s="4" t="s">
         <v>44</v>
@@ -3378,16 +3378,16 @@
         <v>252</v>
       </c>
       <c r="K30" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="L30" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="L30" s="1" t="s">
-        <v>276</v>
-      </c>
       <c r="M30" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="N30" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="31" spans="1:19" ht="116" x14ac:dyDescent="0.35">
@@ -3395,7 +3395,7 @@
         <v>30</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C31" s="4" t="s">
         <v>45</v>
@@ -3410,10 +3410,10 @@
         <v>252</v>
       </c>
       <c r="G31" s="4" t="s">
+        <v>311</v>
+      </c>
+      <c r="J31" s="4" t="s">
         <v>312</v>
-      </c>
-      <c r="J31" s="4" t="s">
-        <v>313</v>
       </c>
       <c r="K31" s="1" t="s">
         <v>249</v>
@@ -3425,10 +3425,10 @@
         <v>253</v>
       </c>
       <c r="N31" s="1" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="P31" s="4" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="32" spans="1:19" ht="29" x14ac:dyDescent="0.35">
@@ -3436,7 +3436,7 @@
         <v>31</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C32" s="4" t="s">
         <v>46</v>
@@ -3451,16 +3451,16 @@
         <v>252</v>
       </c>
       <c r="K32" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="L32" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="L32" s="1" t="s">
-        <v>276</v>
-      </c>
       <c r="M32" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="N32" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="33" spans="1:21" ht="43.5" x14ac:dyDescent="0.35">
@@ -3468,7 +3468,7 @@
         <v>32</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C33" s="4" t="s">
         <v>47</v>
@@ -3480,10 +3480,10 @@
         <v>244</v>
       </c>
       <c r="F33" s="1" t="s">
+        <v>314</v>
+      </c>
+      <c r="G33" s="1" t="s">
         <v>315</v>
-      </c>
-      <c r="G33" s="1" t="s">
-        <v>316</v>
       </c>
       <c r="K33" s="1" t="s">
         <v>249</v>
@@ -3492,16 +3492,16 @@
         <v>250</v>
       </c>
       <c r="M33" s="1" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="N33" s="4" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="O33" s="4" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="P33" s="4" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
     </row>
     <row r="34" spans="1:21" x14ac:dyDescent="0.35">
@@ -3509,7 +3509,7 @@
         <v>33</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C34" s="4" t="s">
         <v>48</v>
@@ -3524,16 +3524,16 @@
         <v>252</v>
       </c>
       <c r="K34" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="L34" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="L34" s="1" t="s">
-        <v>276</v>
-      </c>
       <c r="M34" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="N34" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="35" spans="1:21" ht="29" x14ac:dyDescent="0.35">
@@ -3541,7 +3541,7 @@
         <v>34</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C35" s="4" t="s">
         <v>49</v>
@@ -3556,16 +3556,16 @@
         <v>252</v>
       </c>
       <c r="K35" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="L35" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="L35" s="1" t="s">
-        <v>276</v>
-      </c>
       <c r="M35" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="N35" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="36" spans="1:21" ht="29" x14ac:dyDescent="0.35">
@@ -3573,7 +3573,7 @@
         <v>35</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C36" s="4" t="s">
         <v>50</v>
@@ -3588,16 +3588,16 @@
         <v>252</v>
       </c>
       <c r="K36" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="L36" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="L36" s="1" t="s">
-        <v>276</v>
-      </c>
       <c r="M36" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="N36" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="37" spans="1:21" ht="43.5" x14ac:dyDescent="0.35">
@@ -3605,7 +3605,7 @@
         <v>36</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C37" s="4" t="s">
         <v>51</v>
@@ -3620,16 +3620,16 @@
         <v>252</v>
       </c>
       <c r="K37" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="L37" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="L37" s="1" t="s">
-        <v>276</v>
-      </c>
       <c r="M37" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="N37" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="38" spans="1:21" x14ac:dyDescent="0.35">
@@ -3637,7 +3637,7 @@
         <v>37</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C38" s="4" t="s">
         <v>52</v>
@@ -3652,16 +3652,16 @@
         <v>252</v>
       </c>
       <c r="K38" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="L38" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="L38" s="1" t="s">
-        <v>276</v>
-      </c>
       <c r="M38" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="N38" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="39" spans="1:21" x14ac:dyDescent="0.35">
@@ -3669,7 +3669,7 @@
         <v>38</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C39" s="4" t="s">
         <v>53</v>
@@ -3684,16 +3684,16 @@
         <v>252</v>
       </c>
       <c r="K39" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="L39" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="L39" s="1" t="s">
-        <v>276</v>
-      </c>
       <c r="M39" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="N39" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="40" spans="1:21" ht="43.5" x14ac:dyDescent="0.35">
@@ -3701,7 +3701,7 @@
         <v>39</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C40" s="4" t="s">
         <v>54</v>
@@ -3716,34 +3716,34 @@
         <v>252</v>
       </c>
       <c r="K40" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="L40" s="1" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="M40" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="N40" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="O40" s="4" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="Q40" s="4" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="R40" s="4" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="S40" s="4" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="T40" s="4" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="U40" s="4" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
     </row>
     <row r="41" spans="1:21" ht="43.5" x14ac:dyDescent="0.35">
@@ -3751,7 +3751,7 @@
         <v>40</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C41" s="4" t="s">
         <v>55</v>
@@ -3766,19 +3766,19 @@
         <v>252</v>
       </c>
       <c r="K41" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="L41" s="1" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="M41" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="N41" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="O41" s="4" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
     </row>
     <row r="42" spans="1:21" ht="43.5" x14ac:dyDescent="0.35">
@@ -3786,7 +3786,7 @@
         <v>41</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C42" s="4" t="s">
         <v>56</v>
@@ -3801,34 +3801,34 @@
         <v>252</v>
       </c>
       <c r="K42" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="L42" s="1" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="M42" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="N42" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="O42" s="4" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="Q42" s="4" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="R42" s="4" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="S42" s="4" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="T42" s="4" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="U42" s="4" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
     </row>
     <row r="43" spans="1:21" ht="43.5" x14ac:dyDescent="0.35">
@@ -3836,7 +3836,7 @@
         <v>42</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C43" s="4" t="s">
         <v>57</v>
@@ -3851,19 +3851,19 @@
         <v>252</v>
       </c>
       <c r="K43" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="L43" s="1" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="M43" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="N43" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="O43" s="4" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
     </row>
     <row r="44" spans="1:21" ht="43.5" x14ac:dyDescent="0.35">
@@ -3871,7 +3871,7 @@
         <v>43</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C44" s="4" t="s">
         <v>58</v>
@@ -3886,31 +3886,31 @@
         <v>252</v>
       </c>
       <c r="K44" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="L44" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="L44" s="1" t="s">
-        <v>276</v>
-      </c>
       <c r="M44" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="N44" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="Q44" s="4" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="R44" s="4" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="S44" s="4" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="T44" s="4" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="U44" s="4" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
     </row>
     <row r="45" spans="1:21" ht="362.5" x14ac:dyDescent="0.35">
@@ -3918,7 +3918,7 @@
         <v>44</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C45" s="4" t="s">
         <v>59</v>
@@ -3930,31 +3930,31 @@
         <v>244</v>
       </c>
       <c r="F45" s="4" t="s">
+        <v>320</v>
+      </c>
+      <c r="G45" s="4" t="s">
         <v>321</v>
       </c>
-      <c r="G45" s="4" t="s">
-        <v>322</v>
-      </c>
       <c r="H45" s="4" t="s">
+        <v>317</v>
+      </c>
+      <c r="J45" s="4" t="s">
         <v>318</v>
-      </c>
-      <c r="J45" s="4" t="s">
-        <v>319</v>
       </c>
       <c r="K45" s="1" t="s">
         <v>249</v>
       </c>
       <c r="L45" s="1" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="M45" s="1" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="N45" s="4" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="P45" s="4" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
     </row>
     <row r="46" spans="1:21" ht="174" x14ac:dyDescent="0.35">
@@ -3962,7 +3962,7 @@
         <v>45</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C46" s="4" t="s">
         <v>60</v>
@@ -3974,31 +3974,31 @@
         <v>242</v>
       </c>
       <c r="F46" s="1" t="s">
+        <v>322</v>
+      </c>
+      <c r="G46" s="4" t="s">
         <v>323</v>
       </c>
-      <c r="G46" s="4" t="s">
+      <c r="H46" s="4" t="s">
         <v>324</v>
       </c>
-      <c r="H46" s="4" t="s">
+      <c r="J46" s="4" t="s">
         <v>325</v>
-      </c>
-      <c r="J46" s="4" t="s">
-        <v>326</v>
       </c>
       <c r="K46" s="1" t="s">
         <v>249</v>
       </c>
       <c r="L46" s="1" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="M46" s="1" t="s">
         <v>259</v>
       </c>
       <c r="N46" s="4" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="P46" s="4" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
     </row>
     <row r="47" spans="1:21" ht="43.5" x14ac:dyDescent="0.35">
@@ -4006,7 +4006,7 @@
         <v>46</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C47" s="4" t="s">
         <v>61</v>
@@ -4018,31 +4018,31 @@
         <v>242</v>
       </c>
       <c r="F47" s="1" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="G47" s="4" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="H47" s="4" t="s">
+        <v>330</v>
+      </c>
+      <c r="J47" s="4" t="s">
         <v>331</v>
       </c>
-      <c r="J47" s="4" t="s">
-        <v>332</v>
-      </c>
       <c r="K47" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="L47" s="1" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="M47" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="N47" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="P47" s="4" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
     </row>
     <row r="48" spans="1:21" ht="101.5" x14ac:dyDescent="0.35">
@@ -4050,7 +4050,7 @@
         <v>47</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C48" s="4" t="s">
         <v>62</v>
@@ -4062,16 +4062,16 @@
         <v>242</v>
       </c>
       <c r="F48" s="4" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="G48" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="H48" s="4" t="s">
+        <v>329</v>
+      </c>
+      <c r="J48" s="4" t="s">
         <v>334</v>
-      </c>
-      <c r="H48" s="4" t="s">
-        <v>330</v>
-      </c>
-      <c r="J48" s="4" t="s">
-        <v>335</v>
       </c>
       <c r="K48" s="1" t="s">
         <v>249</v>
@@ -4083,10 +4083,10 @@
         <v>259</v>
       </c>
       <c r="N48" s="4" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="P48" s="4" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
     </row>
     <row r="49" spans="1:16" ht="159.5" x14ac:dyDescent="0.35">
@@ -4094,7 +4094,7 @@
         <v>48</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C49" s="4" t="s">
         <v>63</v>
@@ -4106,28 +4106,28 @@
         <v>244</v>
       </c>
       <c r="F49" s="4" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="G49" s="4" t="s">
+        <v>336</v>
+      </c>
+      <c r="J49" s="4" t="s">
         <v>337</v>
-      </c>
-      <c r="J49" s="4" t="s">
-        <v>338</v>
       </c>
       <c r="K49" s="1" t="s">
         <v>249</v>
       </c>
       <c r="L49" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="M49" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="M49" s="1" t="s">
-        <v>265</v>
-      </c>
       <c r="N49" s="4" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="P49" s="4" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="50" spans="1:16" ht="58" x14ac:dyDescent="0.35">
@@ -4135,7 +4135,7 @@
         <v>49</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C50" s="4" t="s">
         <v>64</v>
@@ -4147,10 +4147,10 @@
         <v>244</v>
       </c>
       <c r="F50" s="1" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="G50" s="4" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="K50" s="1" t="s">
         <v>249</v>
@@ -4159,13 +4159,13 @@
         <v>250</v>
       </c>
       <c r="M50" s="1" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="N50" s="6" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="O50" s="4" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
     </row>
     <row r="51" spans="1:16" ht="261" x14ac:dyDescent="0.35">
@@ -4173,7 +4173,7 @@
         <v>50</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C51" s="4" t="s">
         <v>65</v>
@@ -4185,25 +4185,25 @@
         <v>242</v>
       </c>
       <c r="F51" s="1" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="G51" s="4" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="K51" s="1" t="s">
         <v>249</v>
       </c>
       <c r="L51" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="M51" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="M51" s="1" t="s">
-        <v>265</v>
-      </c>
       <c r="N51" s="4" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="P51" s="4" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
     </row>
     <row r="52" spans="1:16" ht="29" x14ac:dyDescent="0.35">
@@ -4211,7 +4211,7 @@
         <v>51</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C52" s="4" t="s">
         <v>66</v>
@@ -4226,22 +4226,22 @@
         <v>252</v>
       </c>
       <c r="J52" s="4" t="s">
+        <v>431</v>
+      </c>
+      <c r="K52" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="L52" s="1" t="s">
+        <v>275</v>
+      </c>
+      <c r="M52" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="N52" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="P52" s="4" t="s">
         <v>432</v>
-      </c>
-      <c r="K52" s="1" t="s">
-        <v>275</v>
-      </c>
-      <c r="L52" s="1" t="s">
-        <v>276</v>
-      </c>
-      <c r="M52" s="1" t="s">
-        <v>275</v>
-      </c>
-      <c r="N52" s="1" t="s">
-        <v>275</v>
-      </c>
-      <c r="P52" s="4" t="s">
-        <v>433</v>
       </c>
     </row>
     <row r="53" spans="1:16" ht="29" x14ac:dyDescent="0.35">
@@ -4249,7 +4249,7 @@
         <v>52</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C53" s="4" t="s">
         <v>67</v>
@@ -4264,16 +4264,16 @@
         <v>252</v>
       </c>
       <c r="K53" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="L53" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="L53" s="1" t="s">
-        <v>276</v>
-      </c>
       <c r="M53" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="N53" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="54" spans="1:16" ht="29" x14ac:dyDescent="0.35">
@@ -4281,7 +4281,7 @@
         <v>53</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C54" s="4" t="s">
         <v>68</v>
@@ -4296,16 +4296,16 @@
         <v>252</v>
       </c>
       <c r="K54" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="L54" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="L54" s="1" t="s">
-        <v>276</v>
-      </c>
       <c r="M54" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="N54" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="55" spans="1:16" ht="29" x14ac:dyDescent="0.35">
@@ -4313,7 +4313,7 @@
         <v>54</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C55" s="4" t="s">
         <v>69</v>
@@ -4328,16 +4328,16 @@
         <v>252</v>
       </c>
       <c r="K55" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="L55" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="L55" s="1" t="s">
-        <v>276</v>
-      </c>
       <c r="M55" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="N55" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="56" spans="1:16" ht="29" x14ac:dyDescent="0.35">
@@ -4345,7 +4345,7 @@
         <v>55</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C56" s="4" t="s">
         <v>70</v>
@@ -4360,16 +4360,16 @@
         <v>252</v>
       </c>
       <c r="K56" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="L56" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="L56" s="1" t="s">
-        <v>276</v>
-      </c>
       <c r="M56" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="N56" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="57" spans="1:16" ht="29" x14ac:dyDescent="0.35">
@@ -4377,7 +4377,7 @@
         <v>56</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C57" s="4" t="s">
         <v>71</v>
@@ -4392,16 +4392,16 @@
         <v>252</v>
       </c>
       <c r="K57" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="L57" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="L57" s="1" t="s">
-        <v>276</v>
-      </c>
       <c r="M57" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="N57" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="58" spans="1:16" x14ac:dyDescent="0.35">
@@ -4409,7 +4409,7 @@
         <v>57</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C58" s="4" t="s">
         <v>72</v>
@@ -4424,16 +4424,16 @@
         <v>252</v>
       </c>
       <c r="K58" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="L58" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="L58" s="1" t="s">
-        <v>276</v>
-      </c>
       <c r="M58" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="N58" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="59" spans="1:16" ht="29" x14ac:dyDescent="0.35">
@@ -4441,7 +4441,7 @@
         <v>58</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C59" s="4" t="s">
         <v>73</v>
@@ -4456,16 +4456,16 @@
         <v>252</v>
       </c>
       <c r="K59" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="L59" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="L59" s="1" t="s">
-        <v>276</v>
-      </c>
       <c r="M59" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="N59" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="60" spans="1:16" ht="29" x14ac:dyDescent="0.35">
@@ -4473,7 +4473,7 @@
         <v>59</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C60" s="4" t="s">
         <v>74</v>
@@ -4488,16 +4488,16 @@
         <v>252</v>
       </c>
       <c r="K60" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="L60" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="L60" s="1" t="s">
-        <v>276</v>
-      </c>
       <c r="M60" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="N60" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="61" spans="1:16" ht="29" x14ac:dyDescent="0.35">
@@ -4505,7 +4505,7 @@
         <v>60</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C61" s="4" t="s">
         <v>75</v>
@@ -4520,16 +4520,16 @@
         <v>252</v>
       </c>
       <c r="K61" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="L61" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="L61" s="1" t="s">
-        <v>276</v>
-      </c>
       <c r="M61" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="N61" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="62" spans="1:16" ht="29" x14ac:dyDescent="0.35">
@@ -4537,7 +4537,7 @@
         <v>61</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C62" s="4" t="s">
         <v>76</v>
@@ -4552,16 +4552,16 @@
         <v>252</v>
       </c>
       <c r="K62" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="L62" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="L62" s="1" t="s">
-        <v>276</v>
-      </c>
       <c r="M62" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="N62" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="63" spans="1:16" x14ac:dyDescent="0.35">
@@ -4569,7 +4569,7 @@
         <v>62</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C63" s="4" t="s">
         <v>77</v>
@@ -4584,16 +4584,16 @@
         <v>252</v>
       </c>
       <c r="K63" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="L63" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="L63" s="1" t="s">
-        <v>276</v>
-      </c>
       <c r="M63" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="N63" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="64" spans="1:16" x14ac:dyDescent="0.35">
@@ -4601,7 +4601,7 @@
         <v>63</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C64" s="4" t="s">
         <v>78</v>
@@ -4616,16 +4616,16 @@
         <v>252</v>
       </c>
       <c r="K64" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="L64" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="L64" s="1" t="s">
-        <v>276</v>
-      </c>
       <c r="M64" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="N64" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="65" spans="1:17" ht="29" x14ac:dyDescent="0.35">
@@ -4633,7 +4633,7 @@
         <v>64</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C65" s="4" t="s">
         <v>79</v>
@@ -4648,16 +4648,16 @@
         <v>252</v>
       </c>
       <c r="K65" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="L65" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="L65" s="1" t="s">
-        <v>276</v>
-      </c>
       <c r="M65" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="N65" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="66" spans="1:17" ht="58" x14ac:dyDescent="0.35">
@@ -4665,7 +4665,7 @@
         <v>65</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C66" s="4" t="s">
         <v>80</v>
@@ -4680,16 +4680,16 @@
         <v>252</v>
       </c>
       <c r="K66" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="L66" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="L66" s="1" t="s">
-        <v>276</v>
-      </c>
       <c r="M66" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="N66" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="67" spans="1:17" ht="58" x14ac:dyDescent="0.35">
@@ -4697,7 +4697,7 @@
         <v>66</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C67" s="4" t="s">
         <v>81</v>
@@ -4712,16 +4712,16 @@
         <v>252</v>
       </c>
       <c r="K67" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="L67" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="L67" s="1" t="s">
-        <v>276</v>
-      </c>
       <c r="M67" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="N67" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="68" spans="1:17" ht="87" x14ac:dyDescent="0.35">
@@ -4729,7 +4729,7 @@
         <v>67</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C68" s="4" t="s">
         <v>82</v>
@@ -4741,13 +4741,13 @@
         <v>242</v>
       </c>
       <c r="F68" s="1" t="s">
+        <v>340</v>
+      </c>
+      <c r="G68" s="4" t="s">
         <v>341</v>
       </c>
-      <c r="G68" s="4" t="s">
+      <c r="H68" s="4" t="s">
         <v>342</v>
-      </c>
-      <c r="H68" s="4" t="s">
-        <v>343</v>
       </c>
       <c r="K68" s="1" t="s">
         <v>249</v>
@@ -4756,16 +4756,16 @@
         <v>250</v>
       </c>
       <c r="M68" s="1" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="N68" s="1" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="O68" s="5" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="P68" s="4" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="69" spans="1:17" ht="72.5" x14ac:dyDescent="0.35">
@@ -4773,7 +4773,7 @@
         <v>68</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C69" s="4" t="s">
         <v>83</v>
@@ -4785,31 +4785,31 @@
         <v>242</v>
       </c>
       <c r="F69" s="4" t="s">
+        <v>343</v>
+      </c>
+      <c r="G69" s="4" t="s">
         <v>344</v>
       </c>
-      <c r="G69" s="4" t="s">
+      <c r="H69" s="4" t="s">
         <v>345</v>
       </c>
-      <c r="H69" s="4" t="s">
-        <v>346</v>
-      </c>
       <c r="J69" s="4" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="K69" s="1" t="s">
         <v>249</v>
       </c>
       <c r="L69" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="M69" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="M69" s="1" t="s">
-        <v>265</v>
-      </c>
       <c r="N69" s="4" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="P69" s="4" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="Q69" s="5"/>
     </row>
@@ -4818,7 +4818,7 @@
         <v>69</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C70" s="4" t="s">
         <v>84</v>
@@ -4833,16 +4833,16 @@
         <v>252</v>
       </c>
       <c r="K70" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="L70" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="L70" s="1" t="s">
-        <v>276</v>
-      </c>
       <c r="M70" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="N70" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="71" spans="1:17" ht="43.5" x14ac:dyDescent="0.35">
@@ -4850,7 +4850,7 @@
         <v>70</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C71" s="4" t="s">
         <v>85</v>
@@ -4865,16 +4865,16 @@
         <v>252</v>
       </c>
       <c r="K71" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="L71" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="L71" s="1" t="s">
-        <v>276</v>
-      </c>
       <c r="M71" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="N71" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="72" spans="1:17" ht="58" x14ac:dyDescent="0.35">
@@ -4882,7 +4882,7 @@
         <v>71</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C72" s="4" t="s">
         <v>86</v>
@@ -4894,13 +4894,13 @@
         <v>242</v>
       </c>
       <c r="F72" s="4" t="s">
+        <v>349</v>
+      </c>
+      <c r="G72" s="4" t="s">
         <v>350</v>
       </c>
-      <c r="G72" s="4" t="s">
-        <v>351</v>
-      </c>
       <c r="H72" s="4" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="K72" s="1" t="s">
         <v>249</v>
@@ -4912,7 +4912,7 @@
         <v>259</v>
       </c>
       <c r="N72" s="4" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="73" spans="1:17" ht="58" x14ac:dyDescent="0.35">
@@ -4920,7 +4920,7 @@
         <v>72</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C73" s="4" t="s">
         <v>87</v>
@@ -4932,13 +4932,13 @@
         <v>242</v>
       </c>
       <c r="F73" s="4" t="s">
+        <v>351</v>
+      </c>
+      <c r="G73" s="4" t="s">
         <v>352</v>
       </c>
-      <c r="G73" s="4" t="s">
-        <v>353</v>
-      </c>
       <c r="H73" s="4" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="K73" s="1" t="s">
         <v>249</v>
@@ -4950,7 +4950,7 @@
         <v>259</v>
       </c>
       <c r="N73" s="4" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="74" spans="1:17" ht="29" x14ac:dyDescent="0.35">
@@ -4958,7 +4958,7 @@
         <v>73</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C74" s="4" t="s">
         <v>88</v>
@@ -4973,16 +4973,16 @@
         <v>252</v>
       </c>
       <c r="K74" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="L74" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="L74" s="1" t="s">
-        <v>276</v>
-      </c>
       <c r="M74" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="N74" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="75" spans="1:17" ht="29" x14ac:dyDescent="0.35">
@@ -4990,7 +4990,7 @@
         <v>74</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C75" s="4" t="s">
         <v>89</v>
@@ -5005,16 +5005,16 @@
         <v>252</v>
       </c>
       <c r="K75" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="L75" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="L75" s="1" t="s">
-        <v>276</v>
-      </c>
       <c r="M75" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="N75" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="76" spans="1:17" ht="58" x14ac:dyDescent="0.35">
@@ -5022,7 +5022,7 @@
         <v>75</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C76" s="4" t="s">
         <v>90</v>
@@ -5034,13 +5034,13 @@
         <v>242</v>
       </c>
       <c r="F76" s="4" t="s">
+        <v>353</v>
+      </c>
+      <c r="G76" s="4" t="s">
         <v>354</v>
       </c>
-      <c r="G76" s="4" t="s">
-        <v>355</v>
-      </c>
       <c r="H76" s="4" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="K76" s="1" t="s">
         <v>249</v>
@@ -5052,7 +5052,7 @@
         <v>259</v>
       </c>
       <c r="N76" s="4" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="77" spans="1:17" ht="87" x14ac:dyDescent="0.35">
@@ -5060,7 +5060,7 @@
         <v>76</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C77" s="4" t="s">
         <v>91</v>
@@ -5072,31 +5072,31 @@
         <v>242</v>
       </c>
       <c r="F77" s="4" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="G77" s="4" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="H77" s="4" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="K77" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="L77" s="1" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="M77" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="N77" s="4" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="O77" s="4" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="P77" s="4" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="78" spans="1:17" ht="101.5" x14ac:dyDescent="0.35">
@@ -5104,7 +5104,7 @@
         <v>77</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C78" s="4" t="s">
         <v>92</v>
@@ -5116,34 +5116,34 @@
         <v>242</v>
       </c>
       <c r="F78" s="4" t="s">
+        <v>358</v>
+      </c>
+      <c r="G78" s="4" t="s">
         <v>359</v>
       </c>
-      <c r="G78" s="4" t="s">
-        <v>360</v>
-      </c>
       <c r="H78" s="4" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="J78" s="4" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="K78" s="1" t="s">
         <v>249</v>
       </c>
       <c r="L78" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="M78" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="M78" s="1" t="s">
-        <v>265</v>
-      </c>
       <c r="N78" s="4" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="O78" s="4" t="s">
+        <v>437</v>
+      </c>
+      <c r="P78" s="4" t="s">
         <v>438</v>
-      </c>
-      <c r="P78" s="4" t="s">
-        <v>439</v>
       </c>
       <c r="Q78" s="5"/>
     </row>
@@ -5152,7 +5152,7 @@
         <v>78</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C79" s="4" t="s">
         <v>93</v>
@@ -5164,31 +5164,31 @@
         <v>242</v>
       </c>
       <c r="F79" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="G79" s="4" t="s">
         <v>361</v>
       </c>
-      <c r="G79" s="4" t="s">
-        <v>362</v>
-      </c>
       <c r="H79" s="4" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="J79" s="4" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="K79" s="1" t="s">
         <v>249</v>
       </c>
       <c r="L79" s="1" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="M79" s="1" t="s">
         <v>259</v>
       </c>
       <c r="N79" s="4" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="P79" s="4" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
     </row>
     <row r="80" spans="1:17" x14ac:dyDescent="0.35">
@@ -5196,7 +5196,7 @@
         <v>79</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C80" s="4" t="s">
         <v>94</v>
@@ -5211,16 +5211,16 @@
         <v>252</v>
       </c>
       <c r="K80" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="L80" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="L80" s="1" t="s">
-        <v>276</v>
-      </c>
       <c r="M80" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="N80" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="81" spans="1:19" ht="58" x14ac:dyDescent="0.35">
@@ -5228,7 +5228,7 @@
         <v>80</v>
       </c>
       <c r="B81" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C81" s="4" t="s">
         <v>95</v>
@@ -5240,13 +5240,13 @@
         <v>242</v>
       </c>
       <c r="F81" s="1" t="s">
+        <v>362</v>
+      </c>
+      <c r="G81" s="4" t="s">
         <v>363</v>
       </c>
-      <c r="G81" s="4" t="s">
-        <v>364</v>
-      </c>
       <c r="H81" s="4" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="K81" s="1" t="s">
         <v>249</v>
@@ -5258,7 +5258,7 @@
         <v>259</v>
       </c>
       <c r="N81" s="4" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="82" spans="1:19" ht="159.5" x14ac:dyDescent="0.35">
@@ -5266,7 +5266,7 @@
         <v>81</v>
       </c>
       <c r="B82" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C82" s="4" t="s">
         <v>96</v>
@@ -5278,40 +5278,40 @@
         <v>242</v>
       </c>
       <c r="F82" s="1" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="G82" s="4" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="J82" s="4" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="K82" s="1" t="s">
         <v>249</v>
       </c>
       <c r="L82" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="M82" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="M82" s="1" t="s">
-        <v>265</v>
-      </c>
       <c r="N82" s="4" t="s">
+        <v>460</v>
+      </c>
+      <c r="O82" s="4" t="s">
+        <v>408</v>
+      </c>
+      <c r="P82" s="4" t="s">
         <v>461</v>
       </c>
-      <c r="O82" s="4" t="s">
-        <v>409</v>
-      </c>
-      <c r="P82" s="4" t="s">
-        <v>462</v>
-      </c>
       <c r="Q82" s="5" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="R82" s="4" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="S82" s="4" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
     </row>
     <row r="83" spans="1:19" ht="159.5" x14ac:dyDescent="0.35">
@@ -5319,7 +5319,7 @@
         <v>82</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C83" s="4" t="s">
         <v>97</v>
@@ -5331,40 +5331,40 @@
         <v>242</v>
       </c>
       <c r="F83" s="1" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="G83" s="4" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="J83" s="4" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="K83" s="1" t="s">
         <v>249</v>
       </c>
       <c r="L83" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="M83" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="M83" s="1" t="s">
-        <v>265</v>
-      </c>
       <c r="N83" s="4" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="O83" s="4" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="P83" s="4" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="Q83" s="5" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="R83" s="4" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="S83" s="4" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
     </row>
     <row r="84" spans="1:19" ht="159.5" x14ac:dyDescent="0.35">
@@ -5372,7 +5372,7 @@
         <v>83</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C84" s="4" t="s">
         <v>98</v>
@@ -5384,40 +5384,40 @@
         <v>242</v>
       </c>
       <c r="F84" s="1" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="G84" s="4" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="J84" s="4" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="K84" s="1" t="s">
         <v>249</v>
       </c>
       <c r="L84" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="M84" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="M84" s="1" t="s">
-        <v>265</v>
-      </c>
       <c r="N84" s="4" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="O84" s="4" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="P84" s="4" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="Q84" s="5" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="R84" s="4" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="S84" s="4" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
     </row>
     <row r="85" spans="1:19" ht="159.5" x14ac:dyDescent="0.35">
@@ -5425,7 +5425,7 @@
         <v>84</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C85" s="4" t="s">
         <v>99</v>
@@ -5437,40 +5437,40 @@
         <v>242</v>
       </c>
       <c r="F85" s="1" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="G85" s="4" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="J85" s="4" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="K85" s="1" t="s">
         <v>249</v>
       </c>
       <c r="L85" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="M85" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="M85" s="1" t="s">
-        <v>265</v>
-      </c>
       <c r="N85" s="4" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="O85" s="4" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="P85" s="4" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="Q85" s="5" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="R85" s="4" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="S85" s="4" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
     </row>
     <row r="86" spans="1:19" ht="159.5" x14ac:dyDescent="0.35">
@@ -5478,7 +5478,7 @@
         <v>85</v>
       </c>
       <c r="B86" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C86" s="4" t="s">
         <v>100</v>
@@ -5490,40 +5490,40 @@
         <v>242</v>
       </c>
       <c r="F86" s="1" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="G86" s="4" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="J86" s="4" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="K86" s="1" t="s">
         <v>249</v>
       </c>
       <c r="L86" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="M86" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="M86" s="1" t="s">
-        <v>265</v>
-      </c>
       <c r="N86" s="4" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="O86" s="4" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="P86" s="4" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="Q86" s="5" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="R86" s="4" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="S86" s="4" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
     </row>
     <row r="87" spans="1:19" ht="159.5" x14ac:dyDescent="0.35">
@@ -5531,7 +5531,7 @@
         <v>86</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C87" s="4" t="s">
         <v>101</v>
@@ -5543,40 +5543,40 @@
         <v>242</v>
       </c>
       <c r="F87" s="1" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="G87" s="4" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="J87" s="4" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="K87" s="1" t="s">
         <v>249</v>
       </c>
       <c r="L87" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="M87" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="M87" s="1" t="s">
-        <v>265</v>
-      </c>
       <c r="N87" s="4" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="O87" s="4" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="P87" s="4" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="Q87" s="5" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="R87" s="4" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="S87" s="4" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
     </row>
     <row r="88" spans="1:19" ht="159.5" x14ac:dyDescent="0.35">
@@ -5584,7 +5584,7 @@
         <v>87</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C88" s="4" t="s">
         <v>102</v>
@@ -5596,40 +5596,40 @@
         <v>242</v>
       </c>
       <c r="F88" s="1" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="G88" s="4" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="J88" s="4" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="K88" s="1" t="s">
         <v>249</v>
       </c>
       <c r="L88" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="M88" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="M88" s="1" t="s">
-        <v>265</v>
-      </c>
       <c r="N88" s="4" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="O88" s="4" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="P88" s="4" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="Q88" s="5" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="R88" s="4" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="S88" s="4" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
     </row>
     <row r="89" spans="1:19" ht="159.5" x14ac:dyDescent="0.35">
@@ -5637,7 +5637,7 @@
         <v>88</v>
       </c>
       <c r="B89" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C89" s="4" t="s">
         <v>103</v>
@@ -5649,40 +5649,40 @@
         <v>242</v>
       </c>
       <c r="F89" s="1" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="G89" s="4" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="J89" s="4" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="K89" s="1" t="s">
         <v>249</v>
       </c>
       <c r="L89" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="M89" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="M89" s="1" t="s">
-        <v>265</v>
-      </c>
       <c r="N89" s="4" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="O89" s="4" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="P89" s="4" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="Q89" s="5" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="R89" s="4" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="S89" s="4" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
     </row>
     <row r="90" spans="1:19" ht="159.5" x14ac:dyDescent="0.35">
@@ -5690,7 +5690,7 @@
         <v>89</v>
       </c>
       <c r="B90" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C90" s="4" t="s">
         <v>104</v>
@@ -5702,40 +5702,40 @@
         <v>242</v>
       </c>
       <c r="F90" s="1" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="G90" s="4" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="J90" s="4" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="K90" s="1" t="s">
         <v>249</v>
       </c>
       <c r="L90" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="M90" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="M90" s="1" t="s">
-        <v>265</v>
-      </c>
       <c r="N90" s="4" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="O90" s="4" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="P90" s="4" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="Q90" s="5" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="R90" s="4" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="S90" s="4" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
     </row>
     <row r="91" spans="1:19" ht="159.5" x14ac:dyDescent="0.35">
@@ -5743,7 +5743,7 @@
         <v>90</v>
       </c>
       <c r="B91" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C91" s="4" t="s">
         <v>105</v>
@@ -5755,40 +5755,40 @@
         <v>242</v>
       </c>
       <c r="F91" s="1" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="G91" s="4" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="J91" s="4" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="K91" s="1" t="s">
         <v>249</v>
       </c>
       <c r="L91" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="M91" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="M91" s="1" t="s">
-        <v>265</v>
-      </c>
       <c r="N91" s="4" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="O91" s="4" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="P91" s="4" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="Q91" s="5" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="R91" s="13" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="S91" s="4" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
     </row>
     <row r="92" spans="1:19" ht="159.5" x14ac:dyDescent="0.35">
@@ -5796,7 +5796,7 @@
         <v>91</v>
       </c>
       <c r="B92" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C92" s="4" t="s">
         <v>106</v>
@@ -5808,40 +5808,40 @@
         <v>242</v>
       </c>
       <c r="F92" s="1" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="G92" s="4" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="J92" s="4" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="K92" s="1" t="s">
         <v>249</v>
       </c>
       <c r="L92" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="M92" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="M92" s="1" t="s">
-        <v>265</v>
-      </c>
       <c r="N92" s="4" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="O92" s="4" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="P92" s="4" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="Q92" s="5" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="R92" s="13" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="S92" s="4" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
     </row>
     <row r="93" spans="1:19" ht="159.5" x14ac:dyDescent="0.35">
@@ -5849,7 +5849,7 @@
         <v>92</v>
       </c>
       <c r="B93" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C93" s="4" t="s">
         <v>107</v>
@@ -5861,40 +5861,40 @@
         <v>242</v>
       </c>
       <c r="F93" s="1" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="G93" s="4" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="J93" s="4" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="K93" s="1" t="s">
         <v>249</v>
       </c>
       <c r="L93" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="M93" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="M93" s="1" t="s">
-        <v>265</v>
-      </c>
       <c r="N93" s="4" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="O93" s="4" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="P93" s="4" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="Q93" s="5" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="R93" s="13" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="S93" s="4" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
     </row>
     <row r="94" spans="1:19" ht="159.5" x14ac:dyDescent="0.35">
@@ -5902,7 +5902,7 @@
         <v>93</v>
       </c>
       <c r="B94" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C94" s="4" t="s">
         <v>108</v>
@@ -5914,40 +5914,40 @@
         <v>242</v>
       </c>
       <c r="F94" s="1" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="G94" s="4" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="J94" s="4" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="K94" s="1" t="s">
         <v>249</v>
       </c>
       <c r="L94" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="M94" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="M94" s="1" t="s">
-        <v>265</v>
-      </c>
       <c r="N94" s="4" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="O94" s="4" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="P94" s="4" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="Q94" s="5" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="R94" s="13" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="S94" s="4" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
     </row>
     <row r="95" spans="1:19" ht="159.5" x14ac:dyDescent="0.35">
@@ -5955,7 +5955,7 @@
         <v>94</v>
       </c>
       <c r="B95" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C95" s="4" t="s">
         <v>109</v>
@@ -5967,40 +5967,40 @@
         <v>242</v>
       </c>
       <c r="F95" s="1" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="G95" s="4" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="J95" s="4" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="K95" s="1" t="s">
         <v>249</v>
       </c>
       <c r="L95" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="M95" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="M95" s="1" t="s">
-        <v>265</v>
-      </c>
       <c r="N95" s="4" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="O95" s="4" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="P95" s="4" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="Q95" s="5" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="R95" s="13" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="S95" s="4" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
     </row>
     <row r="96" spans="1:19" ht="159.5" x14ac:dyDescent="0.35">
@@ -6008,7 +6008,7 @@
         <v>95</v>
       </c>
       <c r="B96" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C96" s="4" t="s">
         <v>110</v>
@@ -6020,40 +6020,40 @@
         <v>242</v>
       </c>
       <c r="F96" s="1" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="G96" s="4" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="J96" s="4" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="K96" s="1" t="s">
         <v>249</v>
       </c>
       <c r="L96" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="M96" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="M96" s="1" t="s">
-        <v>265</v>
-      </c>
       <c r="N96" s="4" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="O96" s="4" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="P96" s="4" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="Q96" s="5" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="R96" s="13" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="S96" s="4" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
     </row>
     <row r="97" spans="1:19" ht="159.5" x14ac:dyDescent="0.35">
@@ -6061,7 +6061,7 @@
         <v>96</v>
       </c>
       <c r="B97" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C97" s="4" t="s">
         <v>111</v>
@@ -6073,40 +6073,40 @@
         <v>242</v>
       </c>
       <c r="F97" s="1" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="G97" s="4" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="J97" s="4" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="K97" s="1" t="s">
         <v>249</v>
       </c>
       <c r="L97" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="M97" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="M97" s="1" t="s">
-        <v>265</v>
-      </c>
       <c r="N97" s="4" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="O97" s="4" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="P97" s="4" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="Q97" s="5" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="R97" s="13" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="S97" s="4" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
     </row>
     <row r="98" spans="1:19" ht="159.5" x14ac:dyDescent="0.35">
@@ -6114,7 +6114,7 @@
         <v>97</v>
       </c>
       <c r="B98" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C98" s="4" t="s">
         <v>112</v>
@@ -6126,40 +6126,40 @@
         <v>242</v>
       </c>
       <c r="F98" s="1" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="G98" s="4" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="J98" s="4" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="K98" s="1" t="s">
         <v>249</v>
       </c>
       <c r="L98" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="M98" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="M98" s="1" t="s">
-        <v>265</v>
-      </c>
       <c r="N98" s="4" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="O98" s="4" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="P98" s="4" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="Q98" s="5" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="R98" s="13" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="S98" s="4" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
     </row>
     <row r="99" spans="1:19" ht="159.5" x14ac:dyDescent="0.35">
@@ -6167,7 +6167,7 @@
         <v>98</v>
       </c>
       <c r="B99" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C99" s="4" t="s">
         <v>113</v>
@@ -6179,40 +6179,40 @@
         <v>242</v>
       </c>
       <c r="F99" s="1" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="G99" s="4" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="J99" s="4" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="K99" s="1" t="s">
         <v>249</v>
       </c>
       <c r="L99" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="M99" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="M99" s="1" t="s">
-        <v>265</v>
-      </c>
       <c r="N99" s="4" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="O99" s="4" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="P99" s="4" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="Q99" s="5" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="R99" s="13" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="S99" s="4" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
     </row>
     <row r="100" spans="1:19" ht="159.5" x14ac:dyDescent="0.35">
@@ -6220,7 +6220,7 @@
         <v>99</v>
       </c>
       <c r="B100" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C100" s="4" t="s">
         <v>114</v>
@@ -6232,40 +6232,40 @@
         <v>242</v>
       </c>
       <c r="F100" s="1" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="G100" s="4" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="J100" s="4" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="K100" s="1" t="s">
         <v>249</v>
       </c>
       <c r="L100" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="M100" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="M100" s="1" t="s">
-        <v>265</v>
-      </c>
       <c r="N100" s="4" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="O100" s="4" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="P100" s="4" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="Q100" s="5" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="R100" s="13" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="S100" s="4" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
     </row>
     <row r="101" spans="1:19" ht="58" x14ac:dyDescent="0.35">
@@ -6273,7 +6273,7 @@
         <v>100</v>
       </c>
       <c r="B101" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C101" s="4" t="s">
         <v>115</v>
@@ -6285,16 +6285,16 @@
         <v>242</v>
       </c>
       <c r="F101" s="1" t="s">
+        <v>365</v>
+      </c>
+      <c r="G101" s="4" t="s">
         <v>366</v>
       </c>
-      <c r="G101" s="4" t="s">
-        <v>367</v>
-      </c>
       <c r="H101" s="4" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="J101" s="4" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="K101" s="1" t="s">
         <v>249</v>
@@ -6306,7 +6306,7 @@
         <v>259</v>
       </c>
       <c r="N101" s="4" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="102" spans="1:19" x14ac:dyDescent="0.35">
@@ -6314,7 +6314,7 @@
         <v>101</v>
       </c>
       <c r="B102" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C102" s="4" t="s">
         <v>116</v>
@@ -6329,16 +6329,16 @@
         <v>252</v>
       </c>
       <c r="K102" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="L102" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="L102" s="1" t="s">
-        <v>276</v>
-      </c>
       <c r="M102" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="N102" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="103" spans="1:19" x14ac:dyDescent="0.35">
@@ -6346,7 +6346,7 @@
         <v>102</v>
       </c>
       <c r="B103" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C103" s="4" t="s">
         <v>117</v>
@@ -6361,16 +6361,16 @@
         <v>252</v>
       </c>
       <c r="K103" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="L103" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="L103" s="1" t="s">
-        <v>276</v>
-      </c>
       <c r="M103" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="N103" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="104" spans="1:19" ht="87" x14ac:dyDescent="0.35">
@@ -6378,7 +6378,7 @@
         <v>103</v>
       </c>
       <c r="B104" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C104" s="4" t="s">
         <v>118</v>
@@ -6390,28 +6390,28 @@
         <v>242</v>
       </c>
       <c r="F104" s="1" t="s">
+        <v>367</v>
+      </c>
+      <c r="G104" s="4" t="s">
         <v>368</v>
       </c>
-      <c r="G104" s="4" t="s">
+      <c r="I104" s="4" t="s">
         <v>369</v>
       </c>
-      <c r="I104" s="4" t="s">
-        <v>370</v>
-      </c>
       <c r="J104" s="4" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="K104" s="1" t="s">
         <v>249</v>
       </c>
       <c r="L104" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="M104" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="M104" s="1" t="s">
-        <v>265</v>
-      </c>
       <c r="N104" s="4" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
     </row>
     <row r="105" spans="1:19" ht="87" x14ac:dyDescent="0.35">
@@ -6419,7 +6419,7 @@
         <v>104</v>
       </c>
       <c r="B105" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C105" s="4" t="s">
         <v>119</v>
@@ -6431,25 +6431,25 @@
         <v>242</v>
       </c>
       <c r="F105" s="1" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="G105" s="4" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="J105" s="4" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="K105" s="1" t="s">
         <v>249</v>
       </c>
       <c r="L105" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="M105" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="M105" s="1" t="s">
-        <v>265</v>
-      </c>
       <c r="N105" s="4" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
     </row>
     <row r="106" spans="1:19" ht="87" x14ac:dyDescent="0.35">
@@ -6457,7 +6457,7 @@
         <v>105</v>
       </c>
       <c r="B106" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C106" s="4" t="s">
         <v>120</v>
@@ -6469,28 +6469,28 @@
         <v>242</v>
       </c>
       <c r="F106" s="4" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="G106" s="4" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="I106" s="4" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="J106" s="4" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="K106" s="1" t="s">
         <v>249</v>
       </c>
       <c r="L106" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="M106" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="M106" s="1" t="s">
-        <v>265</v>
-      </c>
       <c r="N106" s="4" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
     </row>
     <row r="107" spans="1:19" ht="58" x14ac:dyDescent="0.35">
@@ -6498,7 +6498,7 @@
         <v>106</v>
       </c>
       <c r="B107" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C107" s="4" t="s">
         <v>121</v>
@@ -6513,16 +6513,16 @@
         <v>252</v>
       </c>
       <c r="K107" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="L107" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="L107" s="1" t="s">
-        <v>276</v>
-      </c>
       <c r="M107" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="N107" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="108" spans="1:19" ht="58" x14ac:dyDescent="0.35">
@@ -6530,7 +6530,7 @@
         <v>107</v>
       </c>
       <c r="B108" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C108" s="4" t="s">
         <v>122</v>
@@ -6545,16 +6545,16 @@
         <v>252</v>
       </c>
       <c r="K108" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="L108" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="L108" s="1" t="s">
-        <v>276</v>
-      </c>
       <c r="M108" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="N108" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="109" spans="1:19" ht="29" x14ac:dyDescent="0.35">
@@ -6562,7 +6562,7 @@
         <v>108</v>
       </c>
       <c r="B109" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C109" s="4" t="s">
         <v>123</v>
@@ -6577,16 +6577,16 @@
         <v>252</v>
       </c>
       <c r="K109" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="L109" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="L109" s="1" t="s">
-        <v>276</v>
-      </c>
       <c r="M109" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="N109" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="110" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
@@ -6594,7 +6594,7 @@
         <v>109</v>
       </c>
       <c r="B110" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C110" s="4" t="s">
         <v>124</v>
@@ -6609,16 +6609,16 @@
         <v>252</v>
       </c>
       <c r="K110" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="L110" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="L110" s="1" t="s">
-        <v>276</v>
-      </c>
       <c r="M110" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="N110" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="111" spans="1:19" ht="275.5" x14ac:dyDescent="0.35">
@@ -6626,7 +6626,7 @@
         <v>110</v>
       </c>
       <c r="B111" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C111" s="4" t="s">
         <v>125</v>
@@ -6638,28 +6638,28 @@
         <v>242</v>
       </c>
       <c r="F111" s="4" t="s">
+        <v>377</v>
+      </c>
+      <c r="G111" s="4" t="s">
         <v>378</v>
       </c>
-      <c r="G111" s="4" t="s">
+      <c r="H111" s="4" t="s">
         <v>379</v>
-      </c>
-      <c r="H111" s="4" t="s">
-        <v>380</v>
       </c>
       <c r="K111" s="1" t="s">
         <v>249</v>
       </c>
       <c r="L111" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="M111" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="M111" s="1" t="s">
-        <v>265</v>
-      </c>
       <c r="N111" s="4" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="O111" s="4" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
     </row>
     <row r="112" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
@@ -6667,7 +6667,7 @@
         <v>111</v>
       </c>
       <c r="B112" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C112" s="4" t="s">
         <v>126</v>
@@ -6682,16 +6682,16 @@
         <v>252</v>
       </c>
       <c r="K112" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="L112" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="L112" s="1" t="s">
-        <v>276</v>
-      </c>
       <c r="M112" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="N112" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="113" spans="1:14" ht="43.5" x14ac:dyDescent="0.35">
@@ -6699,7 +6699,7 @@
         <v>112</v>
       </c>
       <c r="B113" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C113" s="4" t="s">
         <v>127</v>
@@ -6714,16 +6714,16 @@
         <v>252</v>
       </c>
       <c r="K113" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="L113" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="L113" s="1" t="s">
-        <v>276</v>
-      </c>
       <c r="M113" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="N113" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
   </sheetData>

</xml_diff>